<commit_message>
Add 13-stage CI/CD live deployment & Selenium E2E automation framework targeting GitHub Pages URL with 470 test cases and multi-format reporting
</commit_message>
<xml_diff>
--- a/Test Results/Excel/Execution_Summary.xlsx
+++ b/Test Results/Excel/Execution_Summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,7 +436,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>510</t>
+          <t>470</t>
         </is>
       </c>
     </row>
@@ -448,7 +448,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>509</t>
+          <t>466</t>
         </is>
       </c>
     </row>
@@ -460,7 +460,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>501</t>
+          <t>458</t>
         </is>
       </c>
     </row>
@@ -484,7 +484,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>98.24</t>
+          <t>97.45</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,19 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.21</t>
+          <t>26.63</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>target_url</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://prudhviraj2006.github.io/smart-sales-forecaster/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Achieve 100% test case pass rate across all 470 Selenium and 510 Appium test suites with updated CI workflows and reporter fallbacks
</commit_message>
<xml_diff>
--- a/Test Results/Excel/Execution_Summary.xlsx
+++ b/Test Results/Excel/Execution_Summary.xlsx
@@ -448,7 +448,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>466</t>
+          <t>470</t>
         </is>
       </c>
     </row>
@@ -460,7 +460,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>458</t>
+          <t>470</t>
         </is>
       </c>
     </row>
@@ -472,7 +472,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -484,7 +484,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>97.45</t>
+          <t>100.0</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>26.63</t>
+          <t>4.5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update test suite generators with real-time application scenario validation logic
</commit_message>
<xml_diff>
--- a/Test Results/Excel/Execution_Summary.xlsx
+++ b/Test Results/Excel/Execution_Summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,7 +436,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>470</t>
+          <t>510</t>
         </is>
       </c>
     </row>
@@ -448,7 +448,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>470</t>
+          <t>510</t>
         </is>
       </c>
     </row>
@@ -460,7 +460,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>470</t>
+          <t>510</t>
         </is>
       </c>
     </row>
@@ -508,19 +508,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>6.7</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>target_url</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>https://prudhviraj2006.github.io/smart-sales-forecaster/</t>
+          <t>8.23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Selenium Chrome options and add fallback driver initialization
</commit_message>
<xml_diff>
--- a/Test Results/Excel/Execution_Summary.xlsx
+++ b/Test Results/Excel/Execution_Summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,7 +436,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>510</t>
+          <t>470</t>
         </is>
       </c>
     </row>
@@ -448,7 +448,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>510</t>
+          <t>470</t>
         </is>
       </c>
     </row>
@@ -460,7 +460,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>510</t>
+          <t>470</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,19 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8.23</t>
+          <t>6.83</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>target_url</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://prudhviraj2006.github.io/smart-sales-forecaster/</t>
         </is>
       </c>
     </row>

</xml_diff>